<commit_message>
Cập nhật Tiên Tân - Châu Sơn
</commit_message>
<xml_diff>
--- a/DSKH.xlsx
+++ b/DSKH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_render\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5912F65-0B7E-4119-B429-B0E509623B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D8ABB3-BDFB-4959-844F-2239E66248F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="843">
   <si>
     <t>STT</t>
   </si>
@@ -2556,6 +2556,15 @@
   </si>
   <si>
     <t>BL004004</t>
+  </si>
+  <si>
+    <t>Ban QLDA Đầu tư xây dựng số 1 tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>2700999373</t>
+  </si>
+  <si>
+    <t>BL057022</t>
   </si>
 </sst>
 </file>
@@ -2999,17 +3008,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E282"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E283"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="90.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.59765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="90.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.75" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3024,7 +3033,7 @@
       </c>
       <c r="E1" s="6"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -3039,7 +3048,7 @@
       </c>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <f>+A2+1</f>
         <v>2</v>
@@ -3055,7 +3064,7 @@
       </c>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <f t="shared" ref="A4:A67" si="0">+A3+1</f>
         <v>3</v>
@@ -3071,7 +3080,7 @@
       </c>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -3087,7 +3096,7 @@
       </c>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -3103,7 +3112,7 @@
       </c>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -3119,7 +3128,7 @@
       </c>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -3135,7 +3144,7 @@
       </c>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -3151,7 +3160,7 @@
       </c>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -3167,7 +3176,7 @@
       </c>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -3183,7 +3192,7 @@
       </c>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -3199,7 +3208,7 @@
       </c>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -3215,7 +3224,7 @@
       </c>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -3231,7 +3240,7 @@
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -3247,7 +3256,7 @@
       </c>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3263,7 +3272,7 @@
       </c>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -3279,7 +3288,7 @@
       </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3295,7 +3304,7 @@
       </c>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -3311,7 +3320,7 @@
       </c>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3327,7 +3336,7 @@
       </c>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3343,7 +3352,7 @@
       </c>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3359,7 +3368,7 @@
       </c>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3375,7 +3384,7 @@
       </c>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3391,7 +3400,7 @@
       </c>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3407,7 +3416,7 @@
       </c>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3423,7 +3432,7 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3439,7 +3448,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3455,7 +3464,7 @@
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3471,7 +3480,7 @@
       </c>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3487,7 +3496,7 @@
       </c>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3503,7 +3512,7 @@
       </c>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3519,7 +3528,7 @@
       </c>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3535,7 +3544,7 @@
       </c>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3551,7 +3560,7 @@
       </c>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3567,7 +3576,7 @@
       </c>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3583,7 +3592,7 @@
       </c>
       <c r="E36" s="3"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3599,7 +3608,7 @@
       </c>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3615,7 +3624,7 @@
       </c>
       <c r="E38" s="3"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3631,7 +3640,7 @@
       </c>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3647,7 +3656,7 @@
       </c>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:5" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -3663,7 +3672,7 @@
       </c>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -3679,7 +3688,7 @@
       </c>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -3695,7 +3704,7 @@
       </c>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -3711,7 +3720,7 @@
       </c>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -3726,7 +3735,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -3741,7 +3750,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -3756,7 +3765,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -3771,7 +3780,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -3786,7 +3795,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -3801,7 +3810,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" ht="33" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3816,7 +3825,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3831,7 +3840,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3846,7 +3855,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3861,7 +3870,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3876,7 +3885,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3891,7 +3900,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3906,7 +3915,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3921,7 +3930,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3936,7 +3945,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3951,7 +3960,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -3966,7 +3975,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -3981,7 +3990,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -3996,7 +4005,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -4011,7 +4020,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -4026,7 +4035,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -4041,7 +4050,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -4056,7 +4065,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <f t="shared" ref="A68:A131" si="1">+A67+1</f>
         <v>67</v>
@@ -4071,7 +4080,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -4086,7 +4095,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -4101,7 +4110,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -4116,7 +4125,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -4131,7 +4140,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -4146,7 +4155,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4161,7 +4170,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4176,7 +4185,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -4191,7 +4200,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -4206,7 +4215,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -4221,7 +4230,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -4236,7 +4245,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -4251,7 +4260,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -4266,7 +4275,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -4281,7 +4290,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
         <f t="shared" si="1"/>
         <v>82</v>
@@ -4296,7 +4305,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
         <f t="shared" si="1"/>
         <v>83</v>
@@ -4311,7 +4320,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
         <f t="shared" si="1"/>
         <v>84</v>
@@ -4326,7 +4335,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
         <f t="shared" si="1"/>
         <v>85</v>
@@ -4341,7 +4350,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
         <f t="shared" si="1"/>
         <v>86</v>
@@ -4356,7 +4365,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -4371,7 +4380,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
         <f t="shared" si="1"/>
         <v>88</v>
@@ -4386,7 +4395,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
         <f t="shared" si="1"/>
         <v>89</v>
@@ -4401,7 +4410,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <f t="shared" si="1"/>
         <v>90</v>
@@ -4416,7 +4425,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -4431,7 +4440,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -4446,7 +4455,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <f t="shared" si="1"/>
         <v>93</v>
@@ -4461,7 +4470,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="8">
         <f t="shared" si="1"/>
         <v>94</v>
@@ -4476,7 +4485,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="8">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -4491,7 +4500,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="8">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -4506,7 +4515,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="8">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -4519,7 +4528,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4532,7 +4541,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="8">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -4545,7 +4554,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="8">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -4560,7 +4569,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -4575,7 +4584,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="8">
         <f t="shared" si="1"/>
         <v>102</v>
@@ -4588,7 +4597,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="8">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -4601,7 +4610,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="8">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -4616,7 +4625,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="8">
         <f t="shared" si="1"/>
         <v>105</v>
@@ -4631,7 +4640,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="8">
         <f t="shared" si="1"/>
         <v>106</v>
@@ -4646,7 +4655,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
         <f t="shared" si="1"/>
         <v>107</v>
@@ -4661,7 +4670,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="8">
         <f t="shared" si="1"/>
         <v>108</v>
@@ -4676,7 +4685,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="8">
         <f t="shared" si="1"/>
         <v>109</v>
@@ -4691,7 +4700,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="8">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -4706,7 +4715,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="8">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -4721,7 +4730,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
         <f t="shared" si="1"/>
         <v>112</v>
@@ -4736,7 +4745,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="8">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -4751,7 +4760,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="8">
         <f t="shared" si="1"/>
         <v>114</v>
@@ -4766,7 +4775,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="8">
         <f t="shared" si="1"/>
         <v>115</v>
@@ -4781,7 +4790,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="8">
         <f t="shared" si="1"/>
         <v>116</v>
@@ -4796,7 +4805,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="8">
         <f t="shared" si="1"/>
         <v>117</v>
@@ -4811,7 +4820,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="8">
         <f t="shared" si="1"/>
         <v>118</v>
@@ -4826,7 +4835,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="8">
         <f t="shared" si="1"/>
         <v>119</v>
@@ -4841,7 +4850,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="8">
         <f t="shared" si="1"/>
         <v>120</v>
@@ -4856,7 +4865,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="8">
         <f t="shared" si="1"/>
         <v>121</v>
@@ -4871,7 +4880,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="8">
         <f t="shared" si="1"/>
         <v>122</v>
@@ -4886,7 +4895,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="8">
         <f t="shared" si="1"/>
         <v>123</v>
@@ -4901,7 +4910,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="8">
         <f t="shared" si="1"/>
         <v>124</v>
@@ -4916,7 +4925,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="8">
         <f t="shared" si="1"/>
         <v>125</v>
@@ -4931,7 +4940,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="8">
         <f t="shared" si="1"/>
         <v>126</v>
@@ -4946,7 +4955,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="8">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -4961,7 +4970,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="8">
         <f t="shared" si="1"/>
         <v>128</v>
@@ -4976,7 +4985,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="8">
         <f t="shared" si="1"/>
         <v>129</v>
@@ -4991,7 +5000,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="8">
         <f t="shared" si="1"/>
         <v>130</v>
@@ -5006,7 +5015,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="8">
         <f t="shared" ref="A132:A195" si="2">+A131+1</f>
         <v>131</v>
@@ -5021,7 +5030,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="8">
         <f t="shared" si="2"/>
         <v>132</v>
@@ -5036,7 +5045,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="8">
         <f t="shared" si="2"/>
         <v>133</v>
@@ -5051,7 +5060,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="8">
         <f t="shared" si="2"/>
         <v>134</v>
@@ -5066,7 +5075,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="8">
         <f t="shared" si="2"/>
         <v>135</v>
@@ -5081,7 +5090,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" ht="33" x14ac:dyDescent="0.25">
       <c r="A137" s="8">
         <f t="shared" si="2"/>
         <v>136</v>
@@ -5096,7 +5105,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="8">
         <f t="shared" si="2"/>
         <v>137</v>
@@ -5111,7 +5120,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="8">
         <f t="shared" si="2"/>
         <v>138</v>
@@ -5126,7 +5135,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="8">
         <f t="shared" si="2"/>
         <v>139</v>
@@ -5141,7 +5150,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="8">
         <f t="shared" si="2"/>
         <v>140</v>
@@ -5156,7 +5165,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="8">
         <f t="shared" si="2"/>
         <v>141</v>
@@ -5171,7 +5180,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="8">
         <f t="shared" si="2"/>
         <v>142</v>
@@ -5186,7 +5195,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="8">
         <f t="shared" si="2"/>
         <v>143</v>
@@ -5201,7 +5210,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="8">
         <f t="shared" si="2"/>
         <v>144</v>
@@ -5216,7 +5225,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="8">
         <f t="shared" si="2"/>
         <v>145</v>
@@ -5231,7 +5240,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="8">
         <f t="shared" si="2"/>
         <v>146</v>
@@ -5244,7 +5253,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="8">
         <f t="shared" si="2"/>
         <v>147</v>
@@ -5259,7 +5268,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="8">
         <f t="shared" si="2"/>
         <v>148</v>
@@ -5274,7 +5283,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="8">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -5289,7 +5298,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="8">
         <f t="shared" si="2"/>
         <v>150</v>
@@ -5304,7 +5313,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="8">
         <f t="shared" si="2"/>
         <v>151</v>
@@ -5319,7 +5328,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="8">
         <f t="shared" si="2"/>
         <v>152</v>
@@ -5334,7 +5343,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="8">
         <f t="shared" si="2"/>
         <v>153</v>
@@ -5349,7 +5358,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="8">
         <f t="shared" si="2"/>
         <v>154</v>
@@ -5364,7 +5373,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="8">
         <f t="shared" si="2"/>
         <v>155</v>
@@ -5379,7 +5388,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="8">
         <f t="shared" si="2"/>
         <v>156</v>
@@ -5394,7 +5403,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="8">
         <f t="shared" si="2"/>
         <v>157</v>
@@ -5409,7 +5418,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="8">
         <f t="shared" si="2"/>
         <v>158</v>
@@ -5424,7 +5433,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="8">
         <f t="shared" si="2"/>
         <v>159</v>
@@ -5439,7 +5448,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="8">
         <f t="shared" si="2"/>
         <v>160</v>
@@ -5454,7 +5463,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="8">
         <f t="shared" si="2"/>
         <v>161</v>
@@ -5469,7 +5478,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="8">
         <f t="shared" si="2"/>
         <v>162</v>
@@ -5484,7 +5493,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="8">
         <f t="shared" si="2"/>
         <v>163</v>
@@ -5499,7 +5508,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="8">
         <f t="shared" si="2"/>
         <v>164</v>
@@ -5514,7 +5523,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="8">
         <f t="shared" si="2"/>
         <v>165</v>
@@ -5529,7 +5538,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="8">
         <f t="shared" si="2"/>
         <v>166</v>
@@ -5544,7 +5553,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="8">
         <f t="shared" si="2"/>
         <v>167</v>
@@ -5559,7 +5568,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="8">
         <f t="shared" si="2"/>
         <v>168</v>
@@ -5574,7 +5583,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="8">
         <f t="shared" si="2"/>
         <v>169</v>
@@ -5589,7 +5598,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="8">
         <f t="shared" si="2"/>
         <v>170</v>
@@ -5604,7 +5613,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="8">
         <f t="shared" si="2"/>
         <v>171</v>
@@ -5619,7 +5628,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="8">
         <f t="shared" si="2"/>
         <v>172</v>
@@ -5634,7 +5643,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="8">
         <f t="shared" si="2"/>
         <v>173</v>
@@ -5649,7 +5658,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="8">
         <f t="shared" si="2"/>
         <v>174</v>
@@ -5664,7 +5673,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="8">
         <f t="shared" si="2"/>
         <v>175</v>
@@ -5679,7 +5688,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="8">
         <f t="shared" si="2"/>
         <v>176</v>
@@ -5694,7 +5703,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="8">
         <f t="shared" si="2"/>
         <v>177</v>
@@ -5709,7 +5718,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="8">
         <f t="shared" si="2"/>
         <v>178</v>
@@ -5724,7 +5733,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="8">
         <f t="shared" si="2"/>
         <v>179</v>
@@ -5739,7 +5748,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="181" spans="1:4" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="8">
         <f t="shared" si="2"/>
         <v>180</v>
@@ -5754,7 +5763,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="8">
         <f t="shared" si="2"/>
         <v>181</v>
@@ -5769,7 +5778,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="8">
         <f t="shared" si="2"/>
         <v>182</v>
@@ -5784,7 +5793,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="8">
         <f t="shared" si="2"/>
         <v>183</v>
@@ -5799,7 +5808,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="8">
         <f t="shared" si="2"/>
         <v>184</v>
@@ -5814,7 +5823,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="8">
         <f t="shared" si="2"/>
         <v>185</v>
@@ -5829,7 +5838,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="8">
         <f t="shared" si="2"/>
         <v>186</v>
@@ -5844,7 +5853,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="8">
         <f t="shared" si="2"/>
         <v>187</v>
@@ -5859,7 +5868,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="8">
         <f t="shared" si="2"/>
         <v>188</v>
@@ -5874,7 +5883,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="8">
         <f t="shared" si="2"/>
         <v>189</v>
@@ -5889,7 +5898,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="8">
         <f t="shared" si="2"/>
         <v>190</v>
@@ -5904,7 +5913,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="8">
         <f t="shared" si="2"/>
         <v>191</v>
@@ -5919,7 +5928,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="8">
         <f t="shared" si="2"/>
         <v>192</v>
@@ -5934,7 +5943,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="8">
         <f t="shared" si="2"/>
         <v>193</v>
@@ -5949,7 +5958,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="8">
         <f t="shared" si="2"/>
         <v>194</v>
@@ -5964,7 +5973,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="8">
         <f t="shared" ref="A196:A259" si="3">+A195+1</f>
         <v>195</v>
@@ -5979,7 +5988,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="8">
         <f t="shared" si="3"/>
         <v>196</v>
@@ -5994,7 +6003,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="8">
         <f t="shared" si="3"/>
         <v>197</v>
@@ -6009,7 +6018,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="8">
         <f t="shared" si="3"/>
         <v>198</v>
@@ -6024,7 +6033,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="8">
         <f t="shared" si="3"/>
         <v>199</v>
@@ -6039,7 +6048,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="8">
         <f t="shared" si="3"/>
         <v>200</v>
@@ -6054,7 +6063,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="8">
         <f t="shared" si="3"/>
         <v>201</v>
@@ -6069,7 +6078,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="8">
         <f t="shared" si="3"/>
         <v>202</v>
@@ -6084,7 +6093,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="8">
         <f t="shared" si="3"/>
         <v>203</v>
@@ -6099,7 +6108,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="8">
         <f t="shared" si="3"/>
         <v>204</v>
@@ -6114,7 +6123,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="8">
         <f t="shared" si="3"/>
         <v>205</v>
@@ -6129,7 +6138,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="8">
         <f t="shared" si="3"/>
         <v>206</v>
@@ -6144,7 +6153,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="8">
         <f t="shared" si="3"/>
         <v>207</v>
@@ -6159,7 +6168,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="8">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -6174,7 +6183,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" s="8">
         <f t="shared" si="3"/>
         <v>209</v>
@@ -6189,7 +6198,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" s="8">
         <f t="shared" si="3"/>
         <v>210</v>
@@ -6204,7 +6213,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="8">
         <f t="shared" si="3"/>
         <v>211</v>
@@ -6219,7 +6228,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="8">
         <f t="shared" si="3"/>
         <v>212</v>
@@ -6234,7 +6243,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" s="8">
         <f t="shared" si="3"/>
         <v>213</v>
@@ -6249,7 +6258,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" s="8">
         <f t="shared" si="3"/>
         <v>214</v>
@@ -6264,7 +6273,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="8">
         <f t="shared" si="3"/>
         <v>215</v>
@@ -6279,7 +6288,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="8">
         <f t="shared" si="3"/>
         <v>216</v>
@@ -6294,7 +6303,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="8">
         <f t="shared" si="3"/>
         <v>217</v>
@@ -6309,7 +6318,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" s="8">
         <f t="shared" si="3"/>
         <v>218</v>
@@ -6324,7 +6333,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" s="8">
         <f t="shared" si="3"/>
         <v>219</v>
@@ -6339,7 +6348,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" s="8">
         <f t="shared" si="3"/>
         <v>220</v>
@@ -6354,7 +6363,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="8">
         <f t="shared" si="3"/>
         <v>221</v>
@@ -6369,7 +6378,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" s="8">
         <f t="shared" si="3"/>
         <v>222</v>
@@ -6384,7 +6393,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" s="8">
         <f t="shared" si="3"/>
         <v>223</v>
@@ -6399,7 +6408,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" s="8">
         <f t="shared" si="3"/>
         <v>224</v>
@@ -6414,7 +6423,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" s="8">
         <f t="shared" si="3"/>
         <v>225</v>
@@ -6429,7 +6438,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" s="8">
         <f t="shared" si="3"/>
         <v>226</v>
@@ -6444,7 +6453,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" s="8">
         <f t="shared" si="3"/>
         <v>227</v>
@@ -6459,7 +6468,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" s="8">
         <f t="shared" si="3"/>
         <v>228</v>
@@ -6474,7 +6483,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" s="8">
         <f t="shared" si="3"/>
         <v>229</v>
@@ -6489,7 +6498,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" s="8">
         <f t="shared" si="3"/>
         <v>230</v>
@@ -6504,7 +6513,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" s="8">
         <f t="shared" si="3"/>
         <v>231</v>
@@ -6519,7 +6528,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" s="8">
         <f t="shared" si="3"/>
         <v>232</v>
@@ -6534,7 +6543,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" s="8">
         <f t="shared" si="3"/>
         <v>233</v>
@@ -6549,7 +6558,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" s="8">
         <f t="shared" si="3"/>
         <v>234</v>
@@ -6564,7 +6573,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" s="8">
         <f t="shared" si="3"/>
         <v>235</v>
@@ -6579,7 +6588,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" s="8">
         <f t="shared" si="3"/>
         <v>236</v>
@@ -6594,7 +6603,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" s="8">
         <f t="shared" si="3"/>
         <v>237</v>
@@ -6609,7 +6618,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" s="8">
         <f t="shared" si="3"/>
         <v>238</v>
@@ -6624,7 +6633,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" s="8">
         <f t="shared" si="3"/>
         <v>239</v>
@@ -6639,7 +6648,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" s="8">
         <f t="shared" si="3"/>
         <v>240</v>
@@ -6654,7 +6663,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" s="8">
         <f t="shared" si="3"/>
         <v>241</v>
@@ -6669,7 +6678,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" s="8">
         <f t="shared" si="3"/>
         <v>242</v>
@@ -6684,7 +6693,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" s="8">
         <f t="shared" si="3"/>
         <v>243</v>
@@ -6699,7 +6708,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" s="8">
         <f t="shared" si="3"/>
         <v>244</v>
@@ -6714,7 +6723,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" s="8">
         <f t="shared" si="3"/>
         <v>245</v>
@@ -6729,7 +6738,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" s="8">
         <f t="shared" si="3"/>
         <v>246</v>
@@ -6744,7 +6753,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" s="8">
         <f t="shared" si="3"/>
         <v>247</v>
@@ -6759,7 +6768,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" s="8">
         <f t="shared" si="3"/>
         <v>248</v>
@@ -6774,7 +6783,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" s="8">
         <f t="shared" si="3"/>
         <v>249</v>
@@ -6789,7 +6798,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" s="8">
         <f t="shared" si="3"/>
         <v>250</v>
@@ -6804,7 +6813,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" s="8">
         <f t="shared" si="3"/>
         <v>251</v>
@@ -6819,7 +6828,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" s="8">
         <f t="shared" si="3"/>
         <v>252</v>
@@ -6834,7 +6843,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" s="8">
         <f t="shared" si="3"/>
         <v>253</v>
@@ -6849,7 +6858,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" s="8">
         <f t="shared" si="3"/>
         <v>254</v>
@@ -6864,7 +6873,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" s="8">
         <f t="shared" si="3"/>
         <v>255</v>
@@ -6879,7 +6888,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" s="8">
         <f t="shared" si="3"/>
         <v>256</v>
@@ -6894,7 +6903,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" s="8">
         <f t="shared" si="3"/>
         <v>257</v>
@@ -6909,7 +6918,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" s="8">
         <f t="shared" si="3"/>
         <v>258</v>
@@ -6924,9 +6933,9 @@
         <v>730</v>
       </c>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" s="8">
-        <f t="shared" ref="A260:A282" si="4">+A259+1</f>
+        <f t="shared" ref="A260:A283" si="4">+A259+1</f>
         <v>259</v>
       </c>
       <c r="B260" s="9" t="s">
@@ -6939,7 +6948,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" s="8">
         <f t="shared" si="4"/>
         <v>260</v>
@@ -6954,7 +6963,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" s="8">
         <f t="shared" si="4"/>
         <v>261</v>
@@ -6969,7 +6978,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" s="8">
         <f t="shared" si="4"/>
         <v>262</v>
@@ -6984,7 +6993,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" s="8">
         <f t="shared" si="4"/>
         <v>263</v>
@@ -6999,7 +7008,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" s="8">
         <f t="shared" si="4"/>
         <v>264</v>
@@ -7014,7 +7023,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="8">
         <f t="shared" si="4"/>
         <v>265</v>
@@ -7029,7 +7038,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="8">
         <f t="shared" si="4"/>
         <v>266</v>
@@ -7042,7 +7051,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="8">
         <f t="shared" si="4"/>
         <v>267</v>
@@ -7057,7 +7066,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" s="8">
         <f t="shared" si="4"/>
         <v>268</v>
@@ -7072,7 +7081,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" s="8">
         <f t="shared" si="4"/>
         <v>269</v>
@@ -7087,7 +7096,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" s="8">
         <f t="shared" si="4"/>
         <v>270</v>
@@ -7102,7 +7111,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" s="8">
         <f t="shared" si="4"/>
         <v>271</v>
@@ -7117,7 +7126,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" s="8">
         <f t="shared" si="4"/>
         <v>272</v>
@@ -7132,7 +7141,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" s="8">
         <f t="shared" si="4"/>
         <v>273</v>
@@ -7147,7 +7156,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" s="8">
         <f t="shared" si="4"/>
         <v>274</v>
@@ -7162,7 +7171,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" s="8">
         <f t="shared" si="4"/>
         <v>275</v>
@@ -7177,7 +7186,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" s="8">
         <f t="shared" si="4"/>
         <v>276</v>
@@ -7192,7 +7201,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" s="8">
         <f t="shared" si="4"/>
         <v>277</v>
@@ -7207,7 +7216,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" s="8">
         <f t="shared" si="4"/>
         <v>278</v>
@@ -7222,7 +7231,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" s="8">
         <f t="shared" si="4"/>
         <v>279</v>
@@ -7237,7 +7246,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" s="8">
         <f t="shared" si="4"/>
         <v>280</v>
@@ -7252,7 +7261,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" s="8">
         <f t="shared" si="4"/>
         <v>281</v>
@@ -7267,12 +7276,27 @@
         <v>839</v>
       </c>
     </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A283" s="8">
+        <f t="shared" si="4"/>
+        <v>282</v>
+      </c>
+      <c r="B283" s="21" t="s">
+        <v>840</v>
+      </c>
+      <c r="C283" s="20" t="s">
+        <v>841</v>
+      </c>
+      <c r="D283" s="21" t="s">
+        <v>842</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="C1:C275 C283:C1048576">
+  <conditionalFormatting sqref="C1:C275 C284:C1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D281:D1048576 D1">
+  <conditionalFormatting sqref="D1 D281:D1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>